<commit_message>
Usar consolidado Excel y actualizar cada 12 horas
</commit_message>
<xml_diff>
--- a/budgets.xlsx
+++ b/budgets.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a.naao\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA98BD3C-920A-4287-8C4D-7C51FD8F157A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01CE96E2-68D7-4AE9-BDB7-92812B617C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FC7CC0E1-1197-4BF7-8906-C93BA600EFD6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FC7CC0E1-1197-4BF7-8906-C93BA600EFD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Budgets" sheetId="1" r:id="rId1"/>
+    <sheet name="Consolidado" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
   <si>
     <t>Budget_Generacion_MWh</t>
   </si>
@@ -48,6 +49,27 @@
   </si>
   <si>
     <t>Budget_PPA_MWh</t>
+  </si>
+  <si>
+    <t>Anio</t>
+  </si>
+  <si>
+    <t>Energia_PPA_MWh</t>
+  </si>
+  <si>
+    <t>Energia_Spot_MWh</t>
+  </si>
+  <si>
+    <t>Ingreso_PPA_USD</t>
+  </si>
+  <si>
+    <t>Ingreso_Spot_USD</t>
+  </si>
+  <si>
+    <t>Fuente</t>
+  </si>
+  <si>
+    <t>Excel consolidado</t>
   </si>
 </sst>
 </file>
@@ -55,9 +77,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -71,16 +93,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F5F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -88,17 +129,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFE6E6E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE6E6E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Millares 10 2 2 5 2" xfId="1" xr:uid="{8A319A50-DD26-44A0-B83C-5213A0DBAA75}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{9038FA99-A957-4D44-876E-985B46EA682C}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -583,4 +648,231 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{655123DA-BA3E-4546-8DBD-7BD97B8797EB}">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.25" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="25.125" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="11" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>3044.9871449729999</v>
+      </c>
+      <c r="D2" s="1">
+        <v>285.51285502700011</v>
+      </c>
+      <c r="E2" s="1">
+        <v>17929.502078943689</v>
+      </c>
+      <c r="F2" s="1">
+        <v>247709.70424355351</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B3" s="3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2709.5287466519994</v>
+      </c>
+      <c r="D3" s="1">
+        <v>359.87125334800066</v>
+      </c>
+      <c r="E3" s="1">
+        <v>27840.514646146967</v>
+      </c>
+      <c r="F3" s="1">
+        <v>220420.16354014014</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B4" s="3">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1">
+        <v>3100.256593736</v>
+      </c>
+      <c r="D4" s="1">
+        <v>171.14340626400008</v>
+      </c>
+      <c r="E4" s="1">
+        <v>9232.7726008996451</v>
+      </c>
+      <c r="F4" s="1">
+        <v>252205.87390042358</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="3">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1311.3032443829995</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1736.9967556170006</v>
+      </c>
+      <c r="E5" s="1">
+        <v>102545.34046460525</v>
+      </c>
+      <c r="F5" s="1">
+        <v>106674.51893055701</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B6" s="3">
+        <v>5</v>
+      </c>
+      <c r="C6" s="1">
+        <v>940.5</v>
+      </c>
+      <c r="D6" s="1">
+        <v>2153.3000000000002</v>
+      </c>
+      <c r="E6" s="1">
+        <v>190976.17700000003</v>
+      </c>
+      <c r="F6" s="1">
+        <v>76509.674999999988</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B7" s="3">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1">
+        <v>830.92076759999998</v>
+      </c>
+      <c r="D7" s="1">
+        <v>2067.3383789999998</v>
+      </c>
+      <c r="E7" s="1">
+        <v>143473.28350260001</v>
+      </c>
+      <c r="F7" s="1">
+        <v>67595.404444259999</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B8" s="3">
+        <v>7</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1431.6</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1260.8427017224003</v>
+      </c>
+      <c r="E8" s="1">
+        <v>65815.989029909295</v>
+      </c>
+      <c r="F8" s="1">
+        <v>119524.28399999999</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B9" s="3">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1">
+        <v>824.56075987860004</v>
+      </c>
+      <c r="D9" s="1">
+        <v>1901.2816432698</v>
+      </c>
+      <c r="E9" s="1">
+        <v>60175.564009489171</v>
+      </c>
+      <c r="F9" s="1">
+        <v>68842.57784226432</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Corregir carga de Excel y consulta automática de API
</commit_message>
<xml_diff>
--- a/budgets.xlsx
+++ b/budgets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a.naao\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01CE96E2-68D7-4AE9-BDB7-92812B617C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD04C566-E47E-48DF-8065-E60EE14561FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FC7CC0E1-1197-4BF7-8906-C93BA600EFD6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FC7CC0E1-1197-4BF7-8906-C93BA600EFD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Budgets" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="10">
   <si>
     <t>Budget_Generacion_MWh</t>
   </si>
@@ -495,153 +495,192 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B121426-6B2E-41A3-A3E2-B37B30CFA4B1}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="22.375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="2" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>3296.7057181449459</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>2544</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
+    <row r="3" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B3" s="3">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="C3">
         <v>2977.6696809051123</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>2298</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
+    <row r="4" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B4" s="3">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="C4">
         <v>3296.7057181449459</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>2544</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5">
+    <row r="5" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="3">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>3190.3603723983347</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>2462</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6">
+    <row r="6" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B6" s="3">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>3296.7057181449459</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>2544</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7">
+    <row r="7" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B7" s="3">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="C7">
         <v>3190.3603723983347</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>2462</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8">
+    <row r="8" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B8" s="3">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="C8">
         <v>3296.7057181449459</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>2544</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9">
+    <row r="9" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B9" s="3">
         <v>8</v>
       </c>
-      <c r="B9">
+      <c r="C9">
         <v>3296.7057181449459</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>2491</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10">
+    <row r="10" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B10">
         <v>9</v>
       </c>
-      <c r="B10">
+      <c r="C10">
         <v>3190.3603723983347</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <v>2411</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11">
+    <row r="11" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B11">
         <v>10</v>
       </c>
-      <c r="B11">
+      <c r="C11">
         <v>3296.7057181449459</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>2491</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12">
+    <row r="12" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B12">
         <v>11</v>
       </c>
-      <c r="B12">
+      <c r="C12">
         <v>3190.3603723983347</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <v>2462</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13">
+    <row r="13" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
+        <v>2026</v>
+      </c>
+      <c r="B13">
         <v>12</v>
       </c>
-      <c r="B13">
+      <c r="C13">
         <v>3296.7057181449459</v>
       </c>
-      <c r="C13">
+      <c r="D13">
         <v>2544</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar generación mensual de proyectos
</commit_message>
<xml_diff>
--- a/budgets.xlsx
+++ b/budgets.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a.naao\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD04C566-E47E-48DF-8065-E60EE14561FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F182C27-C9D7-494F-A26B-2444076FDFAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FC7CC0E1-1197-4BF7-8906-C93BA600EFD6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{FC7CC0E1-1197-4BF7-8906-C93BA600EFD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Budgets" sheetId="1" r:id="rId1"/>
     <sheet name="Consolidado" sheetId="2" r:id="rId2"/>
+    <sheet name="Budgets_Proyectos" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="22">
   <si>
     <t>Budget_Generacion_MWh</t>
   </si>
@@ -71,13 +72,50 @@
   <si>
     <t>Excel consolidado</t>
   </si>
+  <si>
+    <t>Año</t>
+  </si>
+  <si>
+    <t>Proyecto</t>
+  </si>
+  <si>
+    <t>LA QUINTA</t>
+  </si>
+  <si>
+    <t>LA PERLA</t>
+  </si>
+  <si>
+    <t>LA HUERTA</t>
+  </si>
+  <si>
+    <t>CHACAICO</t>
+  </si>
+  <si>
+    <t>SANCLEMENTE</t>
+  </si>
+  <si>
+    <t>TRILALEO</t>
+  </si>
+  <si>
+    <t>COLLANCO</t>
+  </si>
+  <si>
+    <t>MARIA ELENA PFV</t>
+  </si>
+  <si>
+    <t>SAN PEDRO III</t>
+  </si>
+  <si>
+    <t>DOÑA CARMEN</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="172" formatCode="0.0"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -150,7 +188,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -159,6 +197,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="172" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares 10 2 2 5 2" xfId="1" xr:uid="{8A319A50-DD26-44A0-B83C-5213A0DBAA75}"/>
@@ -914,4 +953,1834 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E340EC7-9543-49DC-B847-6040E7D14437}">
+  <dimension ref="A1:T121"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="11" style="1"/>
+    <col min="3" max="3" width="14.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="11" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="4">
+        <v>13274.400382387357</v>
+      </c>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="4">
+        <v>11414.670477321422</v>
+      </c>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="4">
+        <v>5622.8750012700575</v>
+      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="4">
+        <v>2059.2808317604499</v>
+      </c>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B6" s="1">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1528.7064911214525</v>
+      </c>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="4">
+        <v>736.46358865917102</v>
+      </c>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
+      <c r="S7" s="4"/>
+      <c r="T7" s="4"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="4">
+        <v>2695.3096502474996</v>
+      </c>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="4">
+        <v>1417.2481142691302</v>
+      </c>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4"/>
+      <c r="T9" s="4"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1613.7876344241349</v>
+      </c>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4"/>
+      <c r="S10" s="4"/>
+      <c r="T10" s="4"/>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="4">
+        <v>484.1770183724658</v>
+      </c>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
+      <c r="Q11" s="4"/>
+      <c r="R11" s="4"/>
+      <c r="S11" s="4"/>
+      <c r="T11" s="4"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B12" s="1">
+        <v>2</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="4">
+        <v>11545.439062317611</v>
+      </c>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
+      <c r="S12" s="4"/>
+      <c r="T12" s="4"/>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B13" s="1">
+        <v>2</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="4">
+        <v>10530.611428269558</v>
+      </c>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
+      <c r="R13" s="4"/>
+      <c r="S13" s="4"/>
+      <c r="T13" s="4"/>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B14" s="1">
+        <v>2</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="4">
+        <v>5083.3772463492332</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B15" s="1">
+        <v>2</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="4">
+        <v>1698.697535264145</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B16" s="1">
+        <v>2</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="4">
+        <v>1252.4479578403648</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B17" s="1">
+        <v>2</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="4">
+        <v>618.54743360143084</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B18" s="1">
+        <v>2</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="4">
+        <v>2187.423211545</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B19" s="1">
+        <v>2</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="4">
+        <v>1193.6890084076099</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B20" s="1">
+        <v>2</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="4">
+        <v>1353.214274712255</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B21" s="1">
+        <v>2</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="4">
+        <v>395.62138472568984</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B22" s="1">
+        <v>3</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="4">
+        <v>11293.775007387358</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B23" s="1">
+        <v>3</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="4">
+        <v>11296.534898710026</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B24" s="1">
+        <v>3</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D24" s="4">
+        <v>4925.7828890532928</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B25" s="1">
+        <v>3</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="4">
+        <v>1614.7030793736808</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B26" s="1">
+        <v>3</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="4">
+        <v>1095.2112839414174</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B27" s="1">
+        <v>3</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="4">
+        <v>562.65572145524857</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B28" s="1">
+        <v>3</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="4">
+        <v>1897.0800366374999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B29" s="1">
+        <v>3</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="4">
+        <v>1081.1052305764424</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B30" s="1">
+        <v>3</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="4">
+        <v>1261.1295213402525</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B31" s="1">
+        <v>3</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" s="4">
+        <v>385.23146952669532</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B32" s="1">
+        <v>4</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="4">
+        <v>9546.6674006974408</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B33" s="1">
+        <v>4</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="4">
+        <v>10120.507779208338</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B34" s="1">
+        <v>4</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D34" s="4">
+        <v>3868.5181107360372</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B35" s="1">
+        <v>4</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="4">
+        <v>1187.6394175408097</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B36" s="1">
+        <v>4</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="4">
+        <v>723.19260405248997</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B37" s="1">
+        <v>4</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="4">
+        <v>376.92430458809241</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B38" s="1">
+        <v>4</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D38" s="4">
+        <v>1233.3161411999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B39" s="1">
+        <v>4</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39" s="4">
+        <v>691.40473698260257</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B40" s="1">
+        <v>4</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="4">
+        <v>1007.5097647719042</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B41" s="1">
+        <v>4</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41" s="4">
+        <v>289.19617982777504</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B42" s="1">
+        <v>5</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D42" s="4">
+        <v>8158.6379823873567</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B43" s="1">
+        <v>5</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D43" s="4">
+        <v>8602.1435243719043</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B44" s="1">
+        <v>5</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D44" s="4">
+        <v>3088.6225994172423</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B45" s="1">
+        <v>5</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45" s="4">
+        <v>783.29515532616767</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B46" s="1">
+        <v>5</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D46" s="4">
+        <v>466.62344908393499</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B47" s="1">
+        <v>5</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" s="4">
+        <v>233.13028064013383</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B48" s="1">
+        <v>5</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D48" s="4">
+        <v>784.52610092999998</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B49" s="1">
+        <v>5</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D49" s="4">
+        <v>404.33584513607997</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B50" s="1">
+        <v>5</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D50" s="4">
+        <v>714.55272312746877</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B51" s="1">
+        <v>5</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" s="4">
+        <v>254.21477947743932</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B52" s="1">
+        <v>6</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D52" s="4">
+        <v>6969.0980756974404</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B53" s="1">
+        <v>6</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D53" s="4">
+        <v>7678.6713263721995</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B54" s="1">
+        <v>6</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D54" s="4">
+        <v>2605.4432888081915</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B55" s="1">
+        <v>6</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D55" s="4">
+        <v>572.28795049107191</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B56" s="1">
+        <v>6</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" s="4">
+        <v>327.24759102428249</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B57" s="1">
+        <v>6</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D57" s="4">
+        <v>181.25259677758191</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B58" s="1">
+        <v>6</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D58" s="4">
+        <v>537.8628726899999</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B59" s="1">
+        <v>6</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D59" s="4">
+        <v>303.20649096630746</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B60" s="1">
+        <v>6</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D60" s="4">
+        <v>518.62905116554134</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B61" s="1">
+        <v>6</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D61" s="4">
+        <v>221.24863791615843</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B62" s="1">
+        <v>7</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D62" s="4">
+        <v>7979.0822823873559</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B63" s="1">
+        <v>7</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D63" s="4">
+        <v>8590.6001218980236</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B64" s="1">
+        <v>7</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D64" s="4">
+        <v>2964.9190166636322</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B65" s="1">
+        <v>7</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65" s="4">
+        <v>690.55229195767288</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B66" s="1">
+        <v>7</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D66" s="4">
+        <v>397.22477192105077</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B67" s="1">
+        <v>7</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D67" s="4">
+        <v>216.91165767772688</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B68" s="1">
+        <v>7</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D68" s="4">
+        <v>661.41551120806446</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B69" s="1">
+        <v>7</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69" s="4">
+        <v>372.00146761392824</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B70" s="1">
+        <v>7</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D70" s="4">
+        <v>642.5858939752452</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B71" s="1">
+        <v>7</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D71" s="4">
+        <v>766.49227824312004</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B72" s="1">
+        <v>8</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D72" s="4">
+        <v>9658.8731073873569</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B73" s="1">
+        <v>8</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D73" s="4">
+        <v>9956.4362564639323</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B74" s="1">
+        <v>8</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D74" s="4">
+        <v>3829.639957244262</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B75" s="1">
+        <v>8</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D75" s="4">
+        <v>950.71434655224061</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B76" s="1">
+        <v>8</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D76" s="4">
+        <v>549.59479248316495</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B77" s="1">
+        <v>8</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D77" s="4">
+        <v>298.09507151749739</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B78" s="1">
+        <v>8</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D78" s="4">
+        <v>942.97296629250002</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B79" s="1">
+        <v>8</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D79" s="4">
+        <v>542.59058456460002</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B80" s="1">
+        <v>8</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D80" s="4">
+        <v>809.59227800103713</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B81" s="1">
+        <v>8</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D81" s="4">
+        <v>997.42729980464992</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B82" s="1">
+        <v>9</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D82" s="4">
+        <v>11827.33980069744</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B83" s="1">
+        <v>9</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D83" s="4">
+        <v>11411.077656329928</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B84" s="1">
+        <v>9</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D84" s="4">
+        <v>4428.5983382518798</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B85" s="1">
+        <v>9</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D85" s="4">
+        <v>1316.0041734141241</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B86" s="1">
+        <v>9</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D86" s="4">
+        <v>832.19805213509244</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B87" s="1">
+        <v>9</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D87" s="4">
+        <v>413.36820718079389</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B88" s="1">
+        <v>9</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D88" s="4">
+        <v>1436.2994227725001</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B89" s="1">
+        <v>9</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D89" s="4">
+        <v>763.20771754763246</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B90" s="1">
+        <v>9</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D90" s="4">
+        <v>1012.4650121569238</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B91" s="1">
+        <v>9</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D91" s="4">
+        <v>1381.4982190956375</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B92" s="1">
+        <v>10</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D92" s="4">
+        <v>12758.713000650001</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B93" s="1">
+        <v>10</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D93" s="4">
+        <v>12368.553229157238</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B94" s="1">
+        <v>10</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D94" s="4">
+        <v>5186.8614523790347</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B95" s="1">
+        <v>10</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D95" s="4">
+        <v>1644.4185984694534</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B96" s="1">
+        <v>10</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96" s="4">
+        <v>1097.7909702034274</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B97" s="1">
+        <v>10</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D97" s="4">
+        <v>546.565572982817</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B98" s="1">
+        <v>10</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D98" s="4">
+        <v>1962.1717218675003</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B99" s="1">
+        <v>10</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D99" s="4">
+        <v>1048.1662684414348</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B100" s="1">
+        <v>10</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D100" s="4">
+        <v>1239.4882316770409</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B101" s="1">
+        <v>10</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D101" s="4">
+        <v>1880.9655621953625</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B102" s="1">
+        <v>11</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D102" s="4">
+        <v>12305.18995355</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B103" s="1">
+        <v>11</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D103" s="4">
+        <v>12098.423941765028</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B104" s="1">
+        <v>11</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D104" s="4">
+        <v>5420.0324254020716</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B105" s="1">
+        <v>11</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D105" s="4">
+        <v>1798.9613183546599</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B106" s="1">
+        <v>11</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D106" s="4">
+        <v>1302.8254963302149</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B107" s="1">
+        <v>11</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D107" s="4">
+        <v>677.08079646015642</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B108" s="1">
+        <v>11</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D108" s="4">
+        <v>2297.9077825274999</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B109" s="1">
+        <v>11</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D109" s="4">
+        <v>1264.6278112042576</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B110" s="1">
+        <v>11</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D110" s="4">
+        <v>1436.9687874879371</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B111" s="1">
+        <v>11</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D111" s="4">
+        <v>2211.4197751867646</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B112" s="1">
+        <v>12</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D112" s="4">
+        <v>13157.695216349997</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B113" s="1">
+        <v>12</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D113" s="4">
+        <v>12032.468508067526</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B114" s="1">
+        <v>12</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D114" s="4">
+        <v>5934.3436781149167</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B115" s="1">
+        <v>12</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D115" s="4">
+        <v>2028.2531078634242</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B116" s="1">
+        <v>12</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116" s="4">
+        <v>1508.9999834180699</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B117" s="1">
+        <v>12</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D117" s="4">
+        <v>745.77179931096316</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B118" s="1">
+        <v>12</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D118" s="4">
+        <v>2644.7779472399998</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B119" s="1">
+        <v>12</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D119" s="4">
+        <v>1416.8207359674225</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B120" s="1">
+        <v>12</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D120" s="4">
+        <v>1543.5043437384934</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B121" s="1">
+        <v>12</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D121" s="4">
+        <v>2431.8467719313626</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Agregar panel mensual consolidado de proyectos
</commit_message>
<xml_diff>
--- a/budgets.xlsx
+++ b/budgets.xlsx
@@ -8,15 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a.naao\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F182C27-C9D7-494F-A26B-2444076FDFAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{068C78D2-731F-460E-825B-CE6306AFA312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{FC7CC0E1-1197-4BF7-8906-C93BA600EFD6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{FC7CC0E1-1197-4BF7-8906-C93BA600EFD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Budgets" sheetId="1" r:id="rId1"/>
     <sheet name="Consolidado" sheetId="2" r:id="rId2"/>
     <sheet name="Budgets_Proyectos" sheetId="3" r:id="rId3"/>
+    <sheet name="Consolidado_Proyectos" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Consolidado_Proyectos!$C$1:$C$91</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="23">
   <si>
     <t>Budget_Generacion_MWh</t>
   </si>
@@ -108,6 +112,9 @@
   <si>
     <t>DOÑA CARMEN</t>
   </si>
+  <si>
+    <t>Generacion_MWh</t>
+  </si>
 </sst>
 </file>
 
@@ -115,7 +122,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="172" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -197,7 +204,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="172" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares 10 2 2 5 2" xfId="1" xr:uid="{8A319A50-DD26-44A0-B83C-5213A0DBAA75}"/>
@@ -2783,4 +2790,1295 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB91FD77-0D1C-43B3-8B82-AEE9D5CCAC1B}">
+  <dimension ref="A1:D91"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="11" style="1"/>
+    <col min="3" max="3" width="18.75" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.625" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="11" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="3">
+        <v>9218.6405209999994</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="3">
+        <v>7790.0241109999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="3">
+        <v>3589.7859539999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1954.738936</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B6" s="1">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="3">
+        <v>1372.4530520000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="3">
+        <v>638.95142899999996</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="3">
+        <v>1602.5669889999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1220.5800710000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="3">
+        <v>1546.614108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="3">
+        <v>424.77982050000003</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B12" s="1">
+        <v>2</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="1">
+        <v>8404.0595560000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B13" s="1">
+        <v>2</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="1">
+        <v>5297.0222160000003</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B14" s="1">
+        <v>2</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="1">
+        <v>3909.9049599999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B15" s="1">
+        <v>2</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="1">
+        <v>1513.9032540000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B16" s="1">
+        <v>2</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1100.8180480000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B17" s="1">
+        <v>2</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="1">
+        <v>564.61265330000003</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B18" s="1">
+        <v>2</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1277.2678739999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B19" s="1">
+        <v>2</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="1">
+        <v>1017.494247</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B20" s="1">
+        <v>2</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="1">
+        <v>1234.0157019999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B21" s="1">
+        <v>2</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="1">
+        <v>373.07252590000002</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B22" s="1">
+        <v>3</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="1">
+        <v>7641.8999350000004</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B23" s="1">
+        <v>3</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="1">
+        <v>4983.3906710000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B24" s="1">
+        <v>3</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D24" s="1">
+        <v>3865.5261350000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B25" s="1">
+        <v>3</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="1">
+        <v>1446.782991</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B26" s="1">
+        <v>3</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="1">
+        <v>967.40519370000004</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B27" s="1">
+        <v>3</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="1">
+        <v>542.36991479999995</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B28" s="1">
+        <v>3</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="1">
+        <v>1173.509065</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B29" s="1">
+        <v>3</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="1">
+        <v>998.29011760000003</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B30" s="1">
+        <v>3</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="1">
+        <v>803.37878520000004</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B31" s="1">
+        <v>3</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" s="1">
+        <v>339.7966763</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B32" s="1">
+        <v>4</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="1">
+        <v>4891.4351550000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B33" s="1">
+        <v>4</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="1">
+        <v>4497.8570360000003</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B34" s="1">
+        <v>4</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D34" s="1">
+        <v>3115.857544</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B35" s="1">
+        <v>4</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="1">
+        <v>981.13966809999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B36" s="1">
+        <v>4</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="1">
+        <v>665.16069219999997</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B37" s="1">
+        <v>4</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="1">
+        <v>373.04489860000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B38" s="1">
+        <v>4</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D38" s="1">
+        <v>875.25538289999997</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B39" s="1">
+        <v>4</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39" s="1">
+        <v>635.23579789999997</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B40" s="1">
+        <v>4</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="1">
+        <v>843.28953669999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B41" s="1">
+        <v>4</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41" s="1">
+        <v>544.9659838</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B42" s="1">
+        <v>5</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D42" s="1">
+        <v>3629.2002339999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B43" s="1">
+        <v>5</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D43" s="1">
+        <v>3943.0958609999998</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B44" s="1">
+        <v>5</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D44" s="1">
+        <v>2202.723536</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B45" s="1">
+        <v>5</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45" s="1">
+        <v>669.65255669999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B46" s="1">
+        <v>5</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D46" s="1">
+        <v>437.79587370000002</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B47" s="1">
+        <v>5</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" s="1">
+        <v>245.11834239999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B48" s="1">
+        <v>5</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D48" s="1">
+        <v>703.48747639999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B49" s="1">
+        <v>5</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D49" s="1">
+        <v>415.65311050000003</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B50" s="1">
+        <v>5</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D50" s="1">
+        <v>671.37210919999995</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B51" s="1">
+        <v>5</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" s="1">
+        <v>702.20479150000006</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B52" s="1">
+        <v>6</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D52" s="1">
+        <v>3133.1131369999998</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B53" s="1">
+        <v>6</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D53" s="1">
+        <v>3463.9999389999998</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B54" s="1">
+        <v>6</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D54" s="1">
+        <v>2192.3365600000002</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B55" s="1">
+        <v>6</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D55" s="1">
+        <v>430.30418090000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B56" s="1">
+        <v>6</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" s="1">
+        <v>301.66448300000002</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B57" s="1">
+        <v>6</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D57" s="1">
+        <v>172.32080089999999</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B58" s="1">
+        <v>6</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D58" s="1">
+        <v>541.58358729999998</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B59" s="1">
+        <v>6</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D59" s="1">
+        <v>251.04822100000001</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B60" s="1">
+        <v>6</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D60" s="1">
+        <v>473.9406219</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B61" s="1">
+        <v>6</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D61" s="1">
+        <v>603.82259610000006</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B62" s="1">
+        <v>7</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D62" s="1">
+        <v>3321.154869</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B63" s="1">
+        <v>7</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D63" s="1">
+        <v>1646.018039</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B64" s="1">
+        <v>7</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D64" s="1">
+        <v>1929.622779</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B65" s="1">
+        <v>7</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65" s="1">
+        <v>280.67741269999999</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B66" s="1">
+        <v>7</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D66" s="1">
+        <v>211.3355966</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B67" s="1">
+        <v>7</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D67" s="1">
+        <v>123.2081993</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B68" s="1">
+        <v>7</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D68" s="1">
+        <v>372.60926319999999</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B69" s="1">
+        <v>7</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69" s="1">
+        <v>225.87486380000001</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B70" s="1">
+        <v>7</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D70" s="1">
+        <v>324.90541530000002</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B71" s="1">
+        <v>7</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D71" s="1">
+        <v>375.94134969999999</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B72" s="1">
+        <v>8</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D72" s="1">
+        <v>3276.1440859999998</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B73" s="1">
+        <v>8</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D73" s="1">
+        <v>3138.8827809999998</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B74" s="1">
+        <v>8</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D74" s="1">
+        <v>2674.925585</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B75" s="1">
+        <v>8</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D75" s="1">
+        <v>700.83172879999995</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B76" s="1">
+        <v>8</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D76" s="1">
+        <v>438.5244065</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B77" s="1">
+        <v>8</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D77" s="1">
+        <v>270.95186419999999</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B78" s="1">
+        <v>8</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D78" s="1">
+        <v>698.5566986</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B79" s="1">
+        <v>8</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D79" s="1">
+        <v>380.09660739999998</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B80" s="1">
+        <v>8</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D80" s="1">
+        <v>549.20978149999996</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B81" s="1">
+        <v>8</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D81" s="1">
+        <v>723.40544939999995</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B82" s="1">
+        <v>9</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D82" s="1">
+        <v>3117.2851649999998</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B83" s="1">
+        <v>9</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D83" s="1">
+        <v>1438.6737290000001</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B84" s="1">
+        <v>9</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D84" s="1">
+        <v>1196.687995</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B85" s="1">
+        <v>9</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D85" s="1">
+        <v>977.23096139999996</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B86" s="1">
+        <v>9</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D86" s="1">
+        <v>664.26976839999998</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B87" s="1">
+        <v>9</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D87" s="1">
+        <v>340.62975269999998</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B88" s="1">
+        <v>9</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D88" s="1">
+        <v>1009.872658</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B89" s="1">
+        <v>9</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D89" s="1">
+        <v>550.42751880000003</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B90" s="1">
+        <v>9</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D90" s="1">
+        <v>673.31796450000002</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B91" s="1">
+        <v>9</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D91" s="1">
+        <v>752.13981690000003</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="C1:C91" xr:uid="{CB91FD77-0D1C-43B3-8B82-AEE9D5CCAC1B}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>